<commit_message>
Adding article for cluster and stratified sampling
</commit_message>
<xml_diff>
--- a/Quotes.xlsx
+++ b/Quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding_Projects\Personal_Blog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{484FD103-E023-414D-922D-9956FC34E85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9767B3E-1157-4FBF-BBDC-0C098BB004D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4065" yWindow="-15810" windowWidth="29040" windowHeight="15210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,17 +16,30 @@
     <sheet name="Knowledge" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Z_1F027E93_A59B_48CA_AE68_028248C2B726_.wvu.FilterData" localSheetId="0" hidden="1">Knowledge!$A$1:$F$3</definedName>
+    <definedName name="Z_1F027E93_A59B_48CA_AE68_028248C2B726_.wvu.FilterData" localSheetId="0" hidden="1">Knowledge!$A$1:$F$4</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <customWorkbookViews>
     <customWorkbookView name="View -&gt; Group by Pick Count" guid="{1F027E93-A59B-48CA-AE68-028248C2B726}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Domain</t>
   </si>
@@ -139,12 +152,94 @@
   <si>
     <t>The LEGO Method for overcoming procrastination is a productivity strategy based on how modern LEGO sets are packaged: breaking a massive, overwhelming project into small, numbered bags that can be completed one at a time.</t>
   </si>
+  <si>
+    <t>Math and Statistics</t>
+  </si>
+  <si>
+    <t>Cluster vs Stratified sampling</t>
+  </si>
+  <si>
+    <t>Statistics</t>
+  </si>
+  <si>
+    <t>Sampling is the process of selecting a subset of a population to draw conclusions about the whole. It saves time, cost, and effort while making research practical. The key methods include stratified sampling, which takes samples from every group; cluster sampling, which studies selected groups; and multi-stage sampling, which selects samples in multiple steps, from larger groups to smaller units.</t>
+  </si>
+  <si>
+    <t>## Overview
+Sampling is the process of selecting a subset of a population to draw conclusions about the whole. It saves time, cost, and effort while making research practical. The key methods include stratified sampling, which takes samples from every group; cluster sampling, which studies selected groups; and multi-stage sampling, which selects samples in multiple steps, from larger groups to smaller units.
+## Explanation
+Cluster sampling and stratified sampling differ mainly in what you select and why you select it. In stratified sampling, you divide the population into groups and sample from every group, while in cluster sampling, you divide the population into groups and select only some groups for study.
+Imagine XLRI has 1,000 students across different programs and years. You want to survey students about campus life, so you need a way to select a manageable sample.
+### Stratified sampling
+Take some students from every group. Divide the students into **strata**, such as `BM (Business Management)`, `HRM (Human Resource Management)`, and other programs, then randomly select students from each group. This ensures every program is represented in your sample.
+```mermaid
+flowchart TD
+    A["All MBA Students"] --&gt; B["BM"]
+    A --&gt; C["HRM"]
+    A --&gt; D["Other Programs"]
+    B --&gt; E["Randomly Select Students"]
+    C --&gt; F["Randomly Select Students"]
+    D --&gt; G["Randomly Select Students"]
+    E --&gt; H["Final Sample"]
+    F --&gt; H
+    G --&gt; H
+    classDef group fill:#DCEBFA,stroke:#3973AC,color:#163A5C
+    classDef result fill:#DDF3E4,stroke:#39845A,color:#174D2D
+    class B,C,D,E,F,G group
+    class H result
+```
+### Cluster sampling
+Divide the students into clusters, such as year (first year or second year), sections etc. You survey students in those selected sections rather than sampling from every section. Ideally, each cluster reflects the wider population. 
+```mermaid
+flowchart TD
+    A["All MBA Students"] --&gt; B["Section 1"]
+    A --&gt; C["Section 2"]
+    A --&gt; D["Section 3"]
+    A --&gt; E["Section 4"]
+    B --&gt; F["Selected"]
+    D --&gt; F
+    F --&gt; G["Survey All Students in Selected Sections"]
+    G --&gt; H["Final Sample"]
+    classDef group fill:#DCEBFA,stroke:#3973AC,color:#163A5C
+    classDef selected fill:#FBE7C6,stroke:#B7791F,color:#704214
+    classDef result fill:#DDF3E4,stroke:#39845A,color:#174D2D
+    class B,C,D,E group
+    class F,G selected
+    class H result
+```
+### Summary of these methods
+| Basis          | Stratified sampling                         | Cluster sampling                                    |
+| -------------- | ------------------------------------------- | --------------------------------------------------- |
+| Selection      | Some members from every stratum             | Some clusters from the population                   |
+| Groups         | Similar members within each stratum         | Ideally, each cluster reflects the wider population |
+| Main objective | Ensure representation and improve precision | Reduce cost and effort                              |
+| Example        | Students sampled from every program         | A few tutorial sections selected                    |
+&gt; [!tip]
+&gt; Stratified means all groups represented; cluster means some groups selected
+### Cluster Sampling Iteratively
+After creating clusters, we can further create clusters to pinpoint the criteria of people we need. Imagine you want to survey MBA students across India, but you cannot visit every college, so you randomly select 3 states, then 4 colleges in each state, then 2 classes in each college, and finally 10 students from each class. You have selected your sample through four stages, giving you \(3 \times 4 \times 2 \times 10 = 240\) students.
+```mermaid
+flowchart TD
+    A["MBA Students Across India"]
+    A --&gt; B["Stage 1: Select 3 States"]
+    B --&gt; C["Stage 2: Select 4 Colleges per State"]
+    C --&gt; D["Stage 3: Select 2 Classes per College"]
+    D --&gt; E["Stage 4: Select 10 Students per Class"]
+    E --&gt; F["Final Sample: 240 Students"]
+    style A fill:#E5E7EB,stroke:#6B7280,color:#111827
+    style B fill:#DBEAFE,stroke:#2563EB,color:#1E3A8A
+    style C fill:#D1FAE5,stroke:#059669,color:#064E3B
+    style D fill:#FEF3C7,stroke:#D97706,color:#78350F
+    style E fill:#F3E8FF,stroke:#9333EA,color:#581C87
+    style F fill:#DCFCE7,stroke:#16A34A,color:#14532D
+```</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -163,6 +258,12 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -186,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -205,6 +306,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -421,7 +528,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:F3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:F4">
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Domain"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Topic" dataDxfId="3"/>
@@ -766,12 +873,22 @@
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
     </row>
-    <row r="4" spans="1:27" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+    <row r="4" spans="1:27" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>20</v>
+      </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>

</xml_diff>

<commit_message>
Convert excel-to-markdown now shows expected deployment link as well
</commit_message>
<xml_diff>
--- a/Quotes.xlsx
+++ b/Quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding_Projects\Personal_Blog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9767B3E-1157-4FBF-BBDC-0C098BB004D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8CD346-F24A-49FB-90ED-584C6B47DC4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4065" yWindow="-15810" windowWidth="29040" windowHeight="15210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Knowledge" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Z_1F027E93_A59B_48CA_AE68_028248C2B726_.wvu.FilterData" localSheetId="0" hidden="1">Knowledge!$A$1:$F$4</definedName>
+    <definedName name="Z_1F027E93_A59B_48CA_AE68_028248C2B726_.wvu.FilterData" localSheetId="0" hidden="1">Knowledge!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <customWorkbookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Domain</t>
   </si>
@@ -59,100 +59,6 @@
     <t>Pick Count</t>
   </si>
   <si>
-    <t>General Management</t>
-  </si>
-  <si>
-    <t>SLA (Service Level Agreements)</t>
-  </si>
-  <si>
-    <t>Reliability</t>
-  </si>
-  <si>
-    <t>An SLA stands for a Service Level Agreement. It is a formal, binding contract or agreement between a service provider and a customer (or between two internal departments) that defines the exact level of service expected to be delivered</t>
-  </si>
-  <si>
-    <t>Anchored by four core pillars: a defined **scope of services**, measurable **performance metrics** (such as a 99.9% uptime baseline or tier-based helpdesk response deadlines), clearly outlined **provider and customer obligations**, and pre-negotiated **penalties and remedies** (like service credits or termination clauses).
-For complex ecosystems, organizations leverage a **multi-level SLA** to bundle various commitments into a single framework. This structured methodology breaks agreements down into three cohesive layers: **corporate-level policies** that apply globally, **customer-level agreements** customized for specific client groups, and **service-level metrics** tied directly to individual tools or assets. Together, these frameworks establish high accountability, streamline operations, and minimize redundancy across diverse workflows.
-An SLA typically outlines:
-- **Scope of Services:** What is included and what is excluded.
-- **Performance Metrics:** Measurable targets such as system uptime (e.g., 99.9%), response times for support tickets, and resolution deadlines.
-- **Responsibilities:** What both the provider and the customer must do to maintain the service.
-- **Penalties and Remedies:** What happens if the provider fails to meet the agreed standards, such as service credits, fee discounts, or a right to terminate the contract. 
-```mermaid
-mindmap
-  root((Core Components&lt;br&gt;of an SLA))
-    **Scope of Services**
-      What is included
-      What is excluded
-    **Performance Metrics**
-      System uptime targets&lt;br&gt;e.g., 99.9%
-      Support ticket&lt;br&gt;response times
-      Resolution deadlines
-    **Responsibilities**
-      Provider obligations
-      Customer obligations
-      Maintenance protocols
-    **Penalties and Remedies**
-      Service credits
-      Fee discounts
-      Termination rights
-```
-Common Types of SLAs
-- **Customer SLA:** An agreement between a service provider and an external client.
-- **Internal SLA:** An agreement between different teams or departments within the same company (e.g., a sales team and a marketing team).
-- **Multi-Level SLA:** A layered agreement that covers various customer segments, multiple support tiers, or a mix of internal and external stakeholders. 
-### Example 1: Cloud Uptime Example (IT &amp; SaaS)
-An enterprise cloud hosting provider (like Amazon Web Services or Microsoft Azure) signs an agreement with an online retail company.
-- **The Promise:** The cloud server will maintain **99.9% uptime** each month.
-- **The Math:** 99.9% uptime allows for roughly 43.8 minutes of unplanned downtime per month. If the server crashes for 5 hours due to a provider failure, they have breached the SLA.
-- **The Penalty / Remedy:** The agreement states that if uptime drops between 99.0% and 99.8%, the customer gets a **10% service credit** on their next monthly bill. If it drops below 95%, they receive a **50% to 100% refund/credit** for that month.
-### Example 2 : Helpdesk Response &amp; Resolution Example (Internal or B2B IT Support)
-An internal IT department or an external managed service provider (MSP) supports a company's employees. The SLA sets strict reaction times based on how badly a problem hurts the business:
-- **Severity 1 (Critical – e.g., entire office internet is down):**
-    - _Response Time:_ Within **15 minutes** (an engineer must acknowledge and start working).
-    - _Resolution Target:_ Within **4 hours**.
-- **Severity 3 (Low – e.g., a printer isn’t connecting on the 2nd floor):**
-    - _Response Time:_ Within **4 business hours**.
-    - _Resolution Target:_ Within **2 to 5 business days**.
-- **The Remedy:** If Severity 1 issues regularly miss the 4-hour fix window without a valid excuse, the contract allows the client to escalate to senior management or withhold a portion of the monthly retainer.
-### Example 3 : Customer Service / E-Commerce Chatbot Example
-An online banking or retail platform guarantees customer service quality for incoming queries:
-- **First-Response Time:** 95% of live-chat or email queries must receive a human or automated response within **2 minutes**.
-- **First-Contact Resolution (FCR):** At least **75% of customer issues** must be completely solved on the first interaction without needing a callback or transfer.
-- **Abandonment Rate:** Fewer than **3% of callers** should hang up before reaching an agent.
-- **The Remedy:** If the provider misses these metrics for two consecutive quarters, the business can penalize the vendor or put the contract up for re-bidding.
-4. Multi-Level SaaS Tier Example (Corporate, Customer, and Service)
-A software company sells a project-management tool to a large hospital network:
-- **Corporate Level:** Applies to everyone—all users must connect using **TLS 1.2+ encryption** and comply with local data-privacy laws.
-- **Customer Level:** Applies specifically to the Hospital Group—they receive a dedicated Account Manager and **24/7 priority phone support**.
-- **Service Level:** Applies to the specific Radiology Imaging module inside the software—it guarantees a **99.99% uptime** and database search response times under **1 second**.</t>
-  </si>
-  <si>
-    <t>Working with yourself</t>
-  </si>
-  <si>
-    <t>LEGO Method of bagging tasks</t>
-  </si>
-  <si>
-    <t>Productivity</t>
-  </si>
-  <si>
-    <t>When you look at a major project as one giant task (like "Write Master's Thesis" or "Clean the Entire House"), your brain experiences cognitive overload. This triggers anxiety, which leads directly to procrastination. Accept that you cannot build the final structure in a single sitting.
-Divide your massive project into highly specific, sequential phases—just like LEGO bags. Each "bag" should represent a micro-milestone that feels completely manageable.
-Instead of: "Prepare quarterly tax report."
-- Bag 1: Gather all receipts from Q3.
-- Bag 2: Log receipts into the spreadsheet.
-- Bag 3: Calculate total expenses.
-### Open Only One Bag at a Time
-When you sit down to work, your only objective is to finish the current numbered bag. Clear your workspace of everything else. Do not worry about Bag 4 while you are working on Bag 2. This hyper-focus lowers the barrier to entry, making it much easier to simply start.
-### Celebrate the Micro-Builds
-Modern LEGO sets give you a sense of accomplishment quickly; finishing Bag 1 usually rewards you with a completed minifig or the base of a vehicle. In your work, acknowledge the completion of each small bag. This releases dopamine, building the positive momentum you need to open the next bag.
-https://lnkd.in/p/d_qAJzJS</t>
-  </si>
-  <si>
-    <t>The LEGO Method for overcoming procrastination is a productivity strategy based on how modern LEGO sets are packaged: breaking a massive, overwhelming project into small, numbered bags that can be completed one at a time.</t>
-  </si>
-  <si>
     <t>Math and Statistics</t>
   </si>
   <si>
@@ -165,10 +71,7 @@
     <t>Sampling is the process of selecting a subset of a population to draw conclusions about the whole. It saves time, cost, and effort while making research practical. The key methods include stratified sampling, which takes samples from every group; cluster sampling, which studies selected groups; and multi-stage sampling, which selects samples in multiple steps, from larger groups to smaller units.</t>
   </si>
   <si>
-    <t>## Overview
-Sampling is the process of selecting a subset of a population to draw conclusions about the whole. It saves time, cost, and effort while making research practical. The key methods include stratified sampling, which takes samples from every group; cluster sampling, which studies selected groups; and multi-stage sampling, which selects samples in multiple steps, from larger groups to smaller units.
-## Explanation
-Cluster sampling and stratified sampling differ mainly in what you select and why you select it. In stratified sampling, you divide the population into groups and sample from every group, while in cluster sampling, you divide the population into groups and select only some groups for study.
+    <t>Cluster sampling and stratified sampling differ mainly in what you select and why you select it. In stratified sampling, you divide the population into groups and sample from every group, while in cluster sampling, you divide the population into groups and select only some groups for study.
 Imagine XLRI has 1,000 students across different programs and years. You want to survey students about campus life, so you need a way to select a manageable sample.
 ### Stratified sampling
 Take some students from every group. Divide the students into **strata**, such as `BM (Business Management)`, `HRM (Human Resource Management)`, and other programs, then randomly select students from each group. This ensures every program is represented in your sample.
@@ -239,7 +142,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -249,13 +152,6 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -287,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -299,18 +195,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -528,7 +415,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:F4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table1" displayName="Table1" ref="A1:F2">
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Domain"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Topic" dataDxfId="3"/>
@@ -794,24 +681,22 @@
       <c r="AA1" s="1"/>
     </row>
     <row r="2" spans="1:27" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="4">
-        <v>0</v>
-      </c>
+      <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -834,22 +719,12 @@
       <c r="Z2" s="1"/>
       <c r="AA2" s="1"/>
     </row>
-    <row r="3" spans="1:27" ht="293.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>14</v>
-      </c>
+    <row r="3" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -873,22 +748,12 @@
       <c r="Z3" s="1"/>
       <c r="AA3" s="1"/>
     </row>
-    <row r="4" spans="1:27" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>20</v>
-      </c>
+    <row r="4" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -29043,12 +28908,6 @@
       <c r="AA974" s="1"/>
     </row>
     <row r="975" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="A975" s="1"/>
-      <c r="B975" s="1"/>
-      <c r="C975" s="1"/>
-      <c r="D975" s="1"/>
-      <c r="E975" s="1"/>
-      <c r="F975" s="1"/>
       <c r="G975" s="1"/>
       <c r="H975" s="1"/>
       <c r="I975" s="1"/>
@@ -29072,12 +28931,6 @@
       <c r="AA975" s="1"/>
     </row>
     <row r="976" spans="1:27" ht="12.75" x14ac:dyDescent="0.35">
-      <c r="A976" s="1"/>
-      <c r="B976" s="1"/>
-      <c r="C976" s="1"/>
-      <c r="D976" s="1"/>
-      <c r="E976" s="1"/>
-      <c r="F976" s="1"/>
       <c r="G976" s="1"/>
       <c r="H976" s="1"/>
       <c r="I976" s="1"/>
@@ -29659,13 +29512,10 @@
       <autoFilter ref="A1:F23" xr:uid="{5817FDCF-08EC-44F6-84BD-8A54B3224FD6}"/>
     </customSheetView>
   </customSheetViews>
-  <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" display="https://lnkd.in/p/d_qAJzJS" xr:uid="{A9135A7B-4C63-48BD-956F-3AD9FF86D3AC}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>